<commit_message>
[umarciano] update template massive import
</commit_message>
<xml_diff>
--- a/script/templates/IMPORT_RISORSE_UMANE.xlsx
+++ b/script/templates/IMPORT_RISORSE_UMANE.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GZOOM\workspace\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GZOOM\workspace\gzoom-legacy\script\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC2A0F63-F3C9-4B47-B8EB-4A9B9597D69E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02D1E855-49D2-4D23-AF73-855F80199745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}" activeTab="-1"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="77">
   <si>
     <t>Person Code</t>
   </si>
@@ -133,13 +133,16 @@
     <t>Data Source</t>
   </si>
   <si>
+    <t>10000</t>
+  </si>
+  <si>
     <t>Paolo</t>
   </si>
   <si>
-    <t>Rossi</t>
-  </si>
-  <si>
-    <t>RSSPLA60R27F205S</t>
+    <t>Direttore</t>
+  </si>
+  <si>
+    <t>AAABBB60R27F205S</t>
   </si>
   <si>
     <t>DIRETTORE</t>
@@ -151,36 +154,110 @@
     <t/>
   </si>
   <si>
-    <t>BSEA4820</t>
+    <t>UOC001</t>
   </si>
   <si>
     <t>ORGANIZATION_UNIT</t>
   </si>
   <si>
-    <t>UOC Cardiologia con UTIC</t>
+    <t>UOC Test1</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>paolo.rossi@aocardarelli.it</t>
+  </si>
+  <si>
+    <t>paolo.direttore</t>
+  </si>
+  <si>
+    <t>EMPLPERF_VALUTATORE</t>
+  </si>
+  <si>
+    <t>IMPORT_HR</t>
+  </si>
+  <si>
+    <t>10001</t>
+  </si>
+  <si>
+    <t>Marco</t>
+  </si>
+  <si>
+    <t>Medico</t>
+  </si>
+  <si>
+    <t>CCCDDD60R27F205S</t>
+  </si>
+  <si>
+    <t>MEDICO</t>
   </si>
   <si>
     <t>N</t>
   </si>
   <si>
-    <t>paolo.rossi@aocardarelli.it</t>
-  </si>
-  <si>
-    <t>paolo.rossi</t>
+    <t>marco.medico</t>
   </si>
   <si>
     <t>EMPLPERF_VALUTATO</t>
   </si>
   <si>
-    <t>IMPORT_HR</t>
+    <t>10002</t>
+  </si>
+  <si>
+    <t>Anna</t>
+  </si>
+  <si>
+    <t>Caposala</t>
+  </si>
+  <si>
+    <t>EEEFFF60R27F205S</t>
+  </si>
+  <si>
+    <t>CAPOSALA</t>
+  </si>
+  <si>
+    <t>anna.caposala</t>
+  </si>
+  <si>
+    <t>10003</t>
+  </si>
+  <si>
+    <t>Giovanni</t>
+  </si>
+  <si>
+    <t>Infermiere</t>
+  </si>
+  <si>
+    <t>GGGHHH60R27F205S</t>
+  </si>
+  <si>
+    <t>INFERMIERE</t>
+  </si>
+  <si>
+    <t>giovanni.infermiere</t>
+  </si>
+  <si>
+    <t>10004</t>
+  </si>
+  <si>
+    <t>Maria</t>
+  </si>
+  <si>
+    <t>OSS</t>
+  </si>
+  <si>
+    <t>LLLMMM60R27F205S</t>
+  </si>
+  <si>
+    <t>maria.oss</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -206,8 +283,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" applyNumberFormat="1" fontId="0" applyFont="1" fillId="0" applyFill="1" borderId="0" applyBorder="1" xfId="0" applyProtection="1"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -226,46 +304,46 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RisorseUmane" displayName="RisorseUmane" ref="A1:AK2" headerRowCount="1">
-  <autoFilter ref="A1:AK2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="RisorseUmane" displayName="RisorseUmane" ref="A1:AK6">
+  <autoFilter ref="A1:AK6" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="37">
-    <tableColumn id="1" name="Person Code"/>
-    <tableColumn id="2" name="First Name"/>
-    <tableColumn id="3" name="Last Name"/>
-    <tableColumn id="4" name="Fiscal Code"/>
-    <tableColumn id="5" name="Person Role Type"/>
-    <tableColumn id="6" name="Employment Position Type"/>
-    <tableColumn id="7" name="Qualification From Date"/>
-    <tableColumn id="8" name="Employment Amount"/>
-    <tableColumn id="9" name="Employment Start Date"/>
-    <tableColumn id="10" name="Employment End Date"/>
-    <tableColumn id="11" name="Employment Org Code"/>
-    <tableColumn id="12" name="Employment Org Role Type"/>
-    <tableColumn id="13" name="Employment Org Description"/>
-    <tableColumn id="14" name="Employment Org Comments"/>
-    <tableColumn id="15" name="Employment Org From Date"/>
-    <tableColumn id="16" name="Employment Org End Date"/>
-    <tableColumn id="17" name="Evaluator Code"/>
-    <tableColumn id="18" name="Evaluator From Date"/>
-    <tableColumn id="19" name="Allocation Org Code"/>
-    <tableColumn id="20" name="Allocation Org Role Type"/>
-    <tableColumn id="21" name="Allocation Org Description"/>
-    <tableColumn id="22" name="Allocation Org Comments"/>
-    <tableColumn id="23" name="Allocation Org From Date"/>
-    <tableColumn id="24" name="Allocation Org End Date"/>
-    <tableColumn id="25" name="Is Evaluation Manager"/>
-    <tableColumn id="26" name="Approver Code"/>
-    <tableColumn id="27" name="Email"/>
-    <tableColumn id="28" name="Mobile Phone"/>
-    <tableColumn id="29" name="User Login ID"/>
-    <tableColumn id="30" name="Group Profile ID"/>
-    <tableColumn id="31" name="Work Effort Assignment Code"/>
-    <tableColumn id="32" name="Work Effort Date"/>
-    <tableColumn id="33" name="Employment Position Type Date"/>
-    <tableColumn id="34" name="Description"/>
-    <tableColumn id="35" name="Comments"/>
-    <tableColumn id="36" name="Reference Date"/>
-    <tableColumn id="37" name="Data Source"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Person Code"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="First Name"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Last Name"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Fiscal Code"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Person Role Type"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Employment Position Type"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Qualification From Date"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Employment Amount"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Employment Start Date"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Employment End Date"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Employment Org Code"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Employment Org Role Type"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Employment Org Description"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Employment Org Comments"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Employment Org From Date"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Employment Org End Date"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Evaluator Code"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Evaluator From Date"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Allocation Org Code"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Allocation Org Role Type"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Allocation Org Description"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0000-000016000000}" name="Allocation Org Comments"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0000-000017000000}" name="Allocation Org From Date"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Allocation Org End Date"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="Is Evaluation Manager"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="Approver Code"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="Email"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="Mobile Phone"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="User Login ID"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="Group Profile ID"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="Work Effort Assignment Code"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="Work Effort Date"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="Employment Position Type Date"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="Description"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Comments"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Reference Date"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0000-000025000000}" name="Data Source"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -587,278 +665,730 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AK6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.7036190032959" customWidth="1"/>
-    <col min="2" max="2" width="13.1812973022461" customWidth="1"/>
-    <col min="3" max="3" width="12.8835849761963" customWidth="1"/>
-    <col min="4" max="4" width="18.6482810974121" customWidth="1"/>
-    <col min="5" max="5" width="18.8102035522461" customWidth="1"/>
-    <col min="6" max="6" width="27.1328392028809" customWidth="1"/>
-    <col min="7" max="7" width="24.6007518768311" customWidth="1"/>
-    <col min="8" max="8" width="22.4277629852295" customWidth="1"/>
-    <col min="9" max="9" width="24.1966419219971" customWidth="1"/>
-    <col min="10" max="10" width="23.2942981719971" customWidth="1"/>
-    <col min="11" max="11" width="23.5081195831299" customWidth="1"/>
-    <col min="12" max="12" width="27.6147022247314" customWidth="1"/>
-    <col min="13" max="13" width="29.0408573150635" customWidth="1"/>
-    <col min="14" max="14" width="28.5231838226318" customWidth="1"/>
-    <col min="15" max="15" width="28.2633266448975" customWidth="1"/>
-    <col min="16" max="16" width="26.9793796539307" customWidth="1"/>
-    <col min="17" max="17" width="16.9840316772461" customWidth="1"/>
-    <col min="18" max="18" width="21.7392387390137" customWidth="1"/>
-    <col min="19" max="19" width="21.1448383331299" customWidth="1"/>
-    <col min="20" max="20" width="25.2514209747314" customWidth="1"/>
-    <col min="21" max="21" width="26.6775760650635" customWidth="1"/>
-    <col min="22" max="22" width="26.1599025726318" customWidth="1"/>
-    <col min="23" max="23" width="25.9000453948975" customWidth="1"/>
-    <col min="24" max="24" width="24.6160984039307" customWidth="1"/>
-    <col min="25" max="25" width="23.1275386810303" customWidth="1"/>
-    <col min="26" max="26" width="16.8541021347046" customWidth="1"/>
-    <col min="27" max="27" width="25.0086765289307" customWidth="1"/>
-    <col min="28" max="28" width="15.9261827468872" customWidth="1"/>
-    <col min="29" max="29" width="15.2540283203125" customWidth="1"/>
-    <col min="30" max="30" width="21.2888126373291" customWidth="1"/>
-    <col min="31" max="31" width="29.6352577209473" customWidth="1"/>
-    <col min="32" max="32" width="18.5728511810303" customWidth="1"/>
-    <col min="33" max="33" width="31.7796020507813" customWidth="1"/>
-    <col min="34" max="34" width="13.6918077468872" customWidth="1"/>
-    <col min="35" max="35" width="13.1741361618042" customWidth="1"/>
-    <col min="36" max="36" width="17.2346820831299" customWidth="1"/>
-    <col min="37" max="37" width="14.2698383331299" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="2" width="13.21875" customWidth="1"/>
+    <col min="3" max="3" width="12.88671875" customWidth="1"/>
+    <col min="4" max="4" width="20.44140625" customWidth="1"/>
+    <col min="5" max="5" width="18.77734375" customWidth="1"/>
+    <col min="6" max="6" width="27.109375" customWidth="1"/>
+    <col min="7" max="7" width="24.5546875" customWidth="1"/>
+    <col min="8" max="8" width="22.44140625" customWidth="1"/>
+    <col min="9" max="9" width="24.21875" customWidth="1"/>
+    <col min="10" max="10" width="23.33203125" customWidth="1"/>
+    <col min="11" max="11" width="23.5546875" customWidth="1"/>
+    <col min="12" max="12" width="27.6640625" customWidth="1"/>
+    <col min="13" max="13" width="29" customWidth="1"/>
+    <col min="14" max="14" width="28.5546875" customWidth="1"/>
+    <col min="15" max="15" width="28.21875" customWidth="1"/>
+    <col min="16" max="16" width="27" customWidth="1"/>
+    <col min="17" max="17" width="17" customWidth="1"/>
+    <col min="18" max="18" width="21.77734375" customWidth="1"/>
+    <col min="19" max="19" width="21.109375" customWidth="1"/>
+    <col min="20" max="20" width="25.21875" customWidth="1"/>
+    <col min="21" max="21" width="26.6640625" customWidth="1"/>
+    <col min="22" max="22" width="26.109375" customWidth="1"/>
+    <col min="23" max="23" width="25.88671875" customWidth="1"/>
+    <col min="24" max="24" width="24.6640625" customWidth="1"/>
+    <col min="25" max="25" width="23.109375" customWidth="1"/>
+    <col min="26" max="26" width="16.88671875" customWidth="1"/>
+    <col min="27" max="27" width="25" customWidth="1"/>
+    <col min="28" max="28" width="15.88671875" customWidth="1"/>
+    <col min="29" max="29" width="18.5546875" customWidth="1"/>
+    <col min="30" max="30" width="23.5546875" customWidth="1"/>
+    <col min="31" max="31" width="29.6640625" customWidth="1"/>
+    <col min="32" max="32" width="18.5546875" customWidth="1"/>
+    <col min="33" max="33" width="31.77734375" customWidth="1"/>
+    <col min="34" max="34" width="13.6640625" customWidth="1"/>
+    <col min="35" max="35" width="13.21875" customWidth="1"/>
+    <col min="36" max="36" width="17.21875" customWidth="1"/>
+    <col min="37" max="37" width="14.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="0" t="s">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="0" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="0" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="0" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="0" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="0" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="0" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="0" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="0" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="0" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="0" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="0" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="0" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="0" t="s">
+      <c r="X1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="0" t="s">
+      <c r="Y1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="0" t="s">
+      <c r="Z1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="0" t="s">
+      <c r="AA1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="0" t="s">
+      <c r="AB1" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="0" t="s">
+      <c r="AC1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="0" t="s">
+      <c r="AD1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="0" t="s">
+      <c r="AE1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="0" t="s">
+      <c r="AF1" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="0" t="s">
+      <c r="AG1" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="0" t="s">
+      <c r="AH1" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="0" t="s">
+      <c r="AI1" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="0" t="s">
+      <c r="AJ1" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="0" t="s">
+      <c r="AK1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="0">
-        <v>123456</v>
-      </c>
-      <c r="B2" s="0" t="s">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="B2" t="s">
         <v>38</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="C2" t="s">
         <v>39</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="D2" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="G2" s="0" t="s">
+      <c r="E2" t="s">
         <v>41</v>
       </c>
-      <c r="H2" s="0">
+      <c r="F2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H2">
         <v>1</v>
       </c>
-      <c r="I2" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="J2" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="K2" s="0" t="s">
-        <v>43</v>
-      </c>
-      <c r="L2" s="0" t="s">
+      <c r="I2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K2" t="s">
         <v>44</v>
       </c>
-      <c r="M2" s="0" t="s">
+      <c r="L2" t="s">
         <v>45</v>
       </c>
-      <c r="N2" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="O2" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="P2" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q2" s="0">
-        <v>78900</v>
-      </c>
-      <c r="R2" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="S2" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="T2" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="U2" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="V2" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="W2" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="X2" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y2" s="0" t="s">
+      <c r="M2" t="s">
         <v>46</v>
       </c>
-      <c r="Z2" s="0">
-        <v>78900</v>
-      </c>
-      <c r="AA2" s="0" t="s">
+      <c r="N2" t="s">
+        <v>43</v>
+      </c>
+      <c r="O2" t="s">
+        <v>42</v>
+      </c>
+      <c r="P2" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="R2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S2" t="s">
+        <v>43</v>
+      </c>
+      <c r="T2" t="s">
+        <v>43</v>
+      </c>
+      <c r="U2" t="s">
+        <v>43</v>
+      </c>
+      <c r="V2" t="s">
+        <v>43</v>
+      </c>
+      <c r="W2" t="s">
+        <v>43</v>
+      </c>
+      <c r="X2" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y2" t="s">
         <v>47</v>
       </c>
-      <c r="AB2" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="AC2" s="0" t="s">
+      <c r="Z2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AA2" t="s">
         <v>48</v>
       </c>
-      <c r="AD2" s="0" t="s">
+      <c r="AB2" t="s">
+        <v>43</v>
+      </c>
+      <c r="AC2" t="s">
         <v>49</v>
       </c>
-      <c r="AE2" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="AF2" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="AG2" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="AH2" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="AI2" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="AJ2" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="AK2" s="0" t="s">
+      <c r="AD2" t="s">
         <v>50</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>43</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>43</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>43</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3" t="s">
+        <v>42</v>
+      </c>
+      <c r="J3" t="s">
+        <v>43</v>
+      </c>
+      <c r="K3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L3" t="s">
+        <v>45</v>
+      </c>
+      <c r="M3" t="s">
+        <v>46</v>
+      </c>
+      <c r="N3" t="s">
+        <v>43</v>
+      </c>
+      <c r="O3" t="s">
+        <v>42</v>
+      </c>
+      <c r="P3" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R3" t="s">
+        <v>42</v>
+      </c>
+      <c r="S3" t="s">
+        <v>43</v>
+      </c>
+      <c r="T3" t="s">
+        <v>43</v>
+      </c>
+      <c r="U3" t="s">
+        <v>43</v>
+      </c>
+      <c r="V3" t="s">
+        <v>43</v>
+      </c>
+      <c r="W3" t="s">
+        <v>43</v>
+      </c>
+      <c r="X3" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>57</v>
+      </c>
+      <c r="Z3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G4" t="s">
+        <v>42</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4" t="s">
+        <v>42</v>
+      </c>
+      <c r="J4" t="s">
+        <v>43</v>
+      </c>
+      <c r="K4" t="s">
+        <v>44</v>
+      </c>
+      <c r="L4" t="s">
+        <v>45</v>
+      </c>
+      <c r="M4" t="s">
+        <v>46</v>
+      </c>
+      <c r="N4" t="s">
+        <v>43</v>
+      </c>
+      <c r="O4" t="s">
+        <v>42</v>
+      </c>
+      <c r="P4" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R4" t="s">
+        <v>42</v>
+      </c>
+      <c r="S4" t="s">
+        <v>43</v>
+      </c>
+      <c r="T4" t="s">
+        <v>43</v>
+      </c>
+      <c r="U4" t="s">
+        <v>43</v>
+      </c>
+      <c r="V4" t="s">
+        <v>43</v>
+      </c>
+      <c r="W4" t="s">
+        <v>43</v>
+      </c>
+      <c r="X4" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>43</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>65</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>50</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>43</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>43</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>43</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>42</v>
+      </c>
+      <c r="AK4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D5" t="s">
+        <v>69</v>
+      </c>
+      <c r="E5" t="s">
+        <v>70</v>
+      </c>
+      <c r="F5" t="s">
+        <v>70</v>
+      </c>
+      <c r="G5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5" t="s">
+        <v>42</v>
+      </c>
+      <c r="J5" t="s">
+        <v>43</v>
+      </c>
+      <c r="K5" t="s">
+        <v>44</v>
+      </c>
+      <c r="L5" t="s">
+        <v>45</v>
+      </c>
+      <c r="M5" t="s">
+        <v>46</v>
+      </c>
+      <c r="N5" t="s">
+        <v>43</v>
+      </c>
+      <c r="O5" t="s">
+        <v>42</v>
+      </c>
+      <c r="P5" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="R5" t="s">
+        <v>42</v>
+      </c>
+      <c r="S5" t="s">
+        <v>43</v>
+      </c>
+      <c r="T5" t="s">
+        <v>43</v>
+      </c>
+      <c r="U5" t="s">
+        <v>43</v>
+      </c>
+      <c r="V5" t="s">
+        <v>43</v>
+      </c>
+      <c r="W5" t="s">
+        <v>43</v>
+      </c>
+      <c r="X5" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>57</v>
+      </c>
+      <c r="Z5" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>43</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>71</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>59</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>43</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>43</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>43</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:37" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" t="s">
+        <v>75</v>
+      </c>
+      <c r="E6" t="s">
+        <v>74</v>
+      </c>
+      <c r="F6" t="s">
+        <v>74</v>
+      </c>
+      <c r="G6" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6" t="s">
+        <v>42</v>
+      </c>
+      <c r="J6" t="s">
+        <v>43</v>
+      </c>
+      <c r="K6" t="s">
+        <v>44</v>
+      </c>
+      <c r="L6" t="s">
+        <v>45</v>
+      </c>
+      <c r="M6" t="s">
+        <v>46</v>
+      </c>
+      <c r="N6" t="s">
+        <v>43</v>
+      </c>
+      <c r="O6" t="s">
+        <v>42</v>
+      </c>
+      <c r="P6" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q6" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="R6" t="s">
+        <v>42</v>
+      </c>
+      <c r="S6" t="s">
+        <v>43</v>
+      </c>
+      <c r="T6" t="s">
+        <v>43</v>
+      </c>
+      <c r="U6" t="s">
+        <v>43</v>
+      </c>
+      <c r="V6" t="s">
+        <v>43</v>
+      </c>
+      <c r="W6" t="s">
+        <v>43</v>
+      </c>
+      <c r="X6" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>57</v>
+      </c>
+      <c r="Z6" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>48</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>43</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>76</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>59</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>43</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG6" t="s">
+        <v>42</v>
+      </c>
+      <c r="AH6" t="s">
+        <v>43</v>
+      </c>
+      <c r="AI6" t="s">
+        <v>43</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>42</v>
+      </c>
+      <c r="AK6" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
-  <headerFooter/>
-  <tableParts>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>

</xml_diff>